<commit_message>
Update Company Resources KPI section and question wording, count each option
</commit_message>
<xml_diff>
--- a/Data/Check-ins 2024 2025/Mena Report - Copy Tech.xlsx
+++ b/Data/Check-ins 2024 2025/Mena Report - Copy Tech.xlsx
@@ -35,9 +35,6 @@
     <t>Department</t>
   </si>
   <si>
-    <t>E Mail</t>
-  </si>
-  <si>
     <t>Manager Name</t>
   </si>
   <si>
@@ -378,6 +375,9 @@
   </si>
   <si>
     <t>Arletteterz@gmail.com</t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
 </sst>
 </file>
@@ -758,36 +758,36 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="G2" s="3">
         <v>46054</v>
@@ -795,22 +795,22 @@
     </row>
     <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="G3" s="3">
         <v>40057</v>
@@ -818,22 +818,22 @@
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="G4" s="3">
         <v>43102</v>
@@ -841,22 +841,22 @@
     </row>
     <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="G5" s="3">
         <v>41000</v>
@@ -864,22 +864,22 @@
     </row>
     <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="G6" s="3">
         <v>45261</v>
@@ -887,22 +887,22 @@
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="G7" s="3">
         <v>33329</v>
@@ -910,22 +910,22 @@
     </row>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="G8" s="3">
         <v>29860</v>
@@ -933,22 +933,22 @@
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="E9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="G9" s="3">
         <v>41334</v>
@@ -956,22 +956,22 @@
     </row>
     <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="G10" s="3">
         <v>41334</v>
@@ -979,22 +979,22 @@
     </row>
     <row r="11" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="G11" s="3">
         <v>44137</v>
@@ -1002,22 +1002,22 @@
     </row>
     <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="G12" s="3">
         <v>43252</v>
@@ -1025,22 +1025,22 @@
     </row>
     <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="G13" s="3">
         <v>29738</v>
@@ -1048,22 +1048,22 @@
     </row>
     <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="G14" s="3">
         <v>37987</v>
@@ -1071,22 +1071,22 @@
     </row>
     <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="G15" s="3">
         <v>32356</v>
@@ -1094,22 +1094,22 @@
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="G16" s="3">
         <v>35582</v>
@@ -1117,22 +1117,22 @@
     </row>
     <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="E17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="G17" s="3">
         <v>28430</v>
@@ -1140,22 +1140,22 @@
     </row>
     <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="G18" s="3">
         <v>43313</v>
@@ -1163,22 +1163,22 @@
     </row>
     <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G19" s="3">
         <v>41699</v>
@@ -1186,22 +1186,22 @@
     </row>
     <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="E20" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G20" s="3">
         <v>43711</v>
@@ -1209,22 +1209,22 @@
     </row>
     <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="G21" s="3">
         <v>41306</v>
@@ -1232,22 +1232,22 @@
     </row>
     <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E22" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G22" s="3">
         <v>39083</v>
@@ -1255,22 +1255,22 @@
     </row>
     <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="E23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="G23" s="3">
         <v>31717</v>
@@ -1278,22 +1278,22 @@
     </row>
     <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="2" t="s">
+      <c r="E24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="G24" s="3">
         <v>43486</v>
@@ -1301,22 +1301,22 @@
     </row>
     <row r="25" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="E25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="G25" s="3">
         <v>43160</v>
@@ -1324,22 +1324,22 @@
     </row>
     <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="G26" s="3">
         <v>38718</v>
@@ -1347,22 +1347,22 @@
     </row>
     <row r="27" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="E27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="G27" s="3">
         <v>43102</v>
@@ -1370,22 +1370,22 @@
     </row>
     <row r="28" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="G28" s="3">
         <v>39783</v>
@@ -1393,22 +1393,22 @@
     </row>
     <row r="29" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="E29" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G29" s="3">
         <v>39661</v>
@@ -1416,22 +1416,22 @@
     </row>
     <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="E30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="G30" s="3">
         <v>38718</v>
@@ -1439,22 +1439,22 @@
     </row>
     <row r="31" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="E31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="G31" s="3">
         <v>46030</v>
@@ -1462,22 +1462,22 @@
     </row>
     <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="E32" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G32" s="3">
         <v>36220</v>
@@ -1485,22 +1485,22 @@
     </row>
     <row r="33" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="E33" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="G33" s="3">
         <v>45580</v>
@@ -1508,22 +1508,22 @@
     </row>
     <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="G34" s="3">
         <v>39904</v>
@@ -1531,22 +1531,22 @@
     </row>
     <row r="35" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="E35" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G35" s="3">
         <v>43102</v>
@@ -1554,22 +1554,22 @@
     </row>
     <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="G36" s="3">
         <v>37803</v>
@@ -1577,22 +1577,22 @@
     </row>
     <row r="37" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="E37" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G37" s="3">
         <v>29099</v>
@@ -1600,22 +1600,22 @@
     </row>
     <row r="38" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="E38" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G38" s="3">
         <v>38718</v>
@@ -1623,22 +1623,22 @@
     </row>
     <row r="39" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="E39" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G39" s="3">
         <v>42644</v>

</xml_diff>